<commit_message>
Korttexter: stämningstext på alla 83 nätverkskort, längre personbeskrivningar för FC och FS
Samma ton som de tryckta person- och leverantörskorten (torr humor, styrka och svaghet).
Stämningstexten ligger i en egen kolumn så att tryckmallen kan sätta den skild från regeltexten.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/F_FC.xlsx
+++ b/kortdata/F_FC.xlsx
@@ -529,7 +529,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Briljant vid förhandlingsbordet, men otålig med tekniken.</t>
+          <t>Får hyresgäster att skriva på innan kaffet hunnit kallna och vet exakt när motparten är redo att ge sig. På kontorsmarknaden är ingen bättre. En värmepump är däremot en svart låda, och energikalkylen lämnas gärna till någon annan.</t>
         </is>
       </c>
       <c r="I2" s="2" t="n">
@@ -572,7 +572,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Kan energisystemen utan och innan, mindre vass i affären.</t>
+          <t>Kan varje fastighets ventilationsaggregat vid namn och ser energiklassen på långt håll. Förskolor är favoriterna, där finns alltid något att förbättra. I förhandlingsrummet blir det däremot lätt för mycket detaljer och för lite affär.</t>
         </is>
       </c>
       <c r="I3" s="2" t="n">
@@ -615,7 +615,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Tar smällarna utan att blinka.</t>
+          <t>Tar smällarna utan att blinka och har alltid en plan B, helst en plan C också. Lokaler med krångliga hyresgäster är specialiteten. Aldrig spektakulär, aldrig panik, men aldrig heller den som vinner budgivningen.</t>
         </is>
       </c>
       <c r="I4" s="2" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Har sett fler stambyten än någon annan och vet vad som kan vänta.</t>
+          <t>Har varit med om fler stambyten än någon annan och vet vad som väntar bakom kaklet. Hyresrätterna sköts tryggt och utan dramatik. Förutsägbart, stabilt och ärligt talat lite trist, precis som det ska vara.</t>
         </is>
       </c>
       <c r="I5" s="2" t="n">
@@ -701,7 +701,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Har fler kontakter än de andra, i rätt korridorer.</t>
+          <t>Har fler kontakter än de andra, och de sitter i rätt korridorer på kommersiella fastighetsmarknaden. Alltid på väg till nästa lunch. Bostadsaffärer tycker hen är lite för små för att riktigt engagera sig i.</t>
         </is>
       </c>
       <c r="I6" s="2" t="n">
@@ -744,7 +744,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Metodisk och förutseende, bygger alltid in en marginal.</t>
+          <t>Metodisk och förutseende, bygger alltid in en marginal och har aldrig bråttom. Budgeten har en rad för det oväntade, och den är aldrig tom. Tar sällan de stora chanserna, men förlorar heller aldrig huset.</t>
         </is>
       </c>
       <c r="I7" s="2" t="n">

</xml_diff>

<commit_message>
FC Skölden skyddar lokal, kontor och förskola redan som junior
Beslut (Niklas) efter simulering: Skölden väljs av 24 % av kvarteren (förut 7–8 %) och
vinner 22–23 % (förut 17–21 %). F_FC.xlsx: typ och juniortext; regelboken 9.2; BALANS.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/F_FC.xlsx
+++ b/kortdata/F_FC.xlsx
@@ -590,7 +590,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>LOKAL</t>
+          <t>LOKAL, KONTOR, FÖRSKOLA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -600,7 +600,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>En gång per kvartal: ignorera ett händelsekort med minus, varning eller direkt minus på en lokal</t>
+          <t>En gång per kvartal: ignorera ett händelsekort med minus, varning eller direkt minus på en lokal, ett kontor eller en förskola</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Tar smällarna utan att blinka och har alltid en plan B, helst en plan C också. Lokaler med krångliga hyresgäster är specialiteten. Aldrig spektakulär, aldrig panik, men aldrig heller den som vinner budgivningen.</t>
+          <t>Tar smällarna utan att blinka och har alltid en plan B, helst en plan C också. Kommersiella fastigheter med krångliga hyresgäster är specialiteten. Aldrig spektakulär, aldrig panik, men aldrig heller den som vinner budgivningen.</t>
         </is>
       </c>
       <c r="I4" s="2" t="n">

</xml_diff>

<commit_message>
FC Bostadsveteranen: negativ händelse på hyresrätt blir en underhållsvarning
Beslut (Niklas): en gång per kvartal (senior två) får ett negativt händelsekort på en hyresrätt
bli en underhållsvarning i stället (ny fråga till_varning). Straffet på hyresrätter kommer vid
fyra varningar som förut; seniorns 'gratis att röja' utgår. Med slumpvis utdelade FC vinner alla
sex 23–27 %. F_FC.xlsx, regelboken 9.8 och BALANS.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/F_FC.xlsx
+++ b/kortdata/F_FC.xlsx
@@ -643,7 +643,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Underhållsvarningar på hyresrätter ger straff först vid 4, och kostar 1 Mkr mindre att röja</t>
+          <t>En gång per kvartal: gör ett negativt händelsekort på en hyresrätt till en underhållsvarning i stället. Varningar på hyresrätter ger straff först vid 4</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -653,7 +653,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Underhållsvarningar på hyresrätter kostar inget att röja.</t>
+          <t>Två gånger per kvartal.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">

</xml_diff>